<commit_message>
Fix: unificar grupos por mayusculas (evita doble conteo) y blindar TOTALes contra descuadre
</commit_message>
<xml_diff>
--- a/informe-compras-evolti/INFORME DE COMPRAS - MULTICENTRO (TECHOS).xlsx
+++ b/informe-compras-evolti/INFORME DE COMPRAS - MULTICENTRO (TECHOS).xlsx
@@ -1242,7 +1242,7 @@
       <c r="B7" s="26" t="n"/>
       <c r="C7" s="27" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="D7" s="28">
@@ -1306,7 +1306,7 @@
       <c r="B9" s="26" t="n"/>
       <c r="C9" s="27" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="D9" s="28">
@@ -1370,7 +1370,7 @@
       <c r="B11" s="26" t="n"/>
       <c r="C11" s="27" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="D11" s="28">
@@ -1434,7 +1434,7 @@
       <c r="B13" s="26" t="n"/>
       <c r="C13" s="27" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="D13" s="28">
@@ -1465,7 +1465,7 @@
     <row r="14">
       <c r="B14" s="20" t="inlineStr">
         <is>
-          <t>Servicios: viáticos</t>
+          <t>Servicios: Viáticos</t>
         </is>
       </c>
       <c r="C14" s="7" t="n"/>
@@ -1498,7 +1498,7 @@
       <c r="B15" s="26" t="n"/>
       <c r="C15" s="27" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="D15" s="28">
@@ -1562,7 +1562,7 @@
       <c r="B17" s="26" t="n"/>
       <c r="C17" s="27" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="D17" s="28">
@@ -1610,7 +1610,7 @@
       <c r="B19" s="26" t="n"/>
       <c r="C19" s="27" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="D19" s="28">
@@ -1658,7 +1658,7 @@
       <c r="B21" s="26" t="n"/>
       <c r="C21" s="27" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="D21" s="28">
@@ -1802,7 +1802,7 @@
       <c r="B27" s="26" t="n"/>
       <c r="C27" s="27" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="D27" s="28">
@@ -1850,7 +1850,7 @@
       <c r="B29" s="26" t="n"/>
       <c r="C29" s="27" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="D29" s="28">
@@ -1878,11 +1878,11 @@
       </c>
       <c r="C30" s="30" t="n"/>
       <c r="D30" s="31">
-        <f>D6+D8+D10+D12+D14+D16+D18+D20+D22+D26+D28</f>
+        <f>SUM(Detalle!$K$2:$K$214)</f>
         <v/>
       </c>
       <c r="E30" s="31">
-        <f>E6+E8+E10+E12+E14+E16+E18+E20+E22+E26+E28</f>
+        <f>SUM(Detalle!$M$2:$M$214)</f>
         <v/>
       </c>
       <c r="F30" s="31">
@@ -2552,11 +2552,11 @@
         <v/>
       </c>
       <c r="D28" s="31">
-        <f>SUM(D7:D27)</f>
+        <f>SUM(Detalle!$K$2:$K$214)</f>
         <v/>
       </c>
       <c r="E28" s="31">
-        <f>SUM(E7:E27)</f>
+        <f>SUM(Detalle!$M$2:$M$214)</f>
         <v/>
       </c>
       <c r="F28" s="31">
@@ -7490,11 +7490,11 @@
         </is>
       </c>
       <c r="C30" s="21">
-        <f>SUM(C6:C29)</f>
+        <f>SUM(Detalle!$K$2:$K$214)</f>
         <v/>
       </c>
       <c r="D30" s="21">
-        <f>SUM(D6:D29)</f>
+        <f>SUM(Detalle!$M$2:$M$214)</f>
         <v/>
       </c>
       <c r="E30" s="21">
@@ -7855,7 +7855,7 @@
       </c>
       <c r="G2" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H2" s="16" t="inlineStr">
@@ -7938,7 +7938,7 @@
       </c>
       <c r="G3" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H3" s="18" t="inlineStr">
@@ -8016,12 +8016,12 @@
       </c>
       <c r="F4" s="16" t="inlineStr">
         <is>
-          <t>Servicios: viáticos</t>
+          <t>Servicios: Viáticos</t>
         </is>
       </c>
       <c r="G4" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H4" s="16" t="inlineStr">
@@ -8099,12 +8099,12 @@
       </c>
       <c r="F5" s="18" t="inlineStr">
         <is>
-          <t>Servicios: viáticos</t>
+          <t>Servicios: Viáticos</t>
         </is>
       </c>
       <c r="G5" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H5" s="18" t="inlineStr">
@@ -8191,7 +8191,7 @@
       </c>
       <c r="G6" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H6" s="16" t="inlineStr">
@@ -8274,7 +8274,7 @@
       </c>
       <c r="G7" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H7" s="18" t="inlineStr">
@@ -8352,12 +8352,12 @@
       </c>
       <c r="F8" s="16" t="inlineStr">
         <is>
-          <t>Servicios: viáticos</t>
+          <t>Servicios: Viáticos</t>
         </is>
       </c>
       <c r="G8" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H8" s="16" t="inlineStr">
@@ -8444,7 +8444,7 @@
       </c>
       <c r="G9" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H9" s="18" t="inlineStr">
@@ -8527,7 +8527,7 @@
       </c>
       <c r="G10" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H10" s="16" t="inlineStr">
@@ -8609,12 +8609,12 @@
       </c>
       <c r="F11" s="18" t="inlineStr">
         <is>
-          <t>Servicios: viáticos</t>
+          <t>Servicios: Viáticos</t>
         </is>
       </c>
       <c r="G11" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H11" s="18" t="inlineStr">
@@ -8692,12 +8692,12 @@
       </c>
       <c r="F12" s="16" t="inlineStr">
         <is>
-          <t>Servicios: viáticos</t>
+          <t>Servicios: Viáticos</t>
         </is>
       </c>
       <c r="G12" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H12" s="16" t="inlineStr">
@@ -8780,7 +8780,7 @@
       </c>
       <c r="G13" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H13" s="18" t="inlineStr">
@@ -8867,7 +8867,7 @@
       </c>
       <c r="G14" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H14" s="16" t="inlineStr">
@@ -8950,7 +8950,7 @@
       </c>
       <c r="G15" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H15" s="18" t="inlineStr">
@@ -9028,12 +9028,12 @@
       </c>
       <c r="F16" s="16" t="inlineStr">
         <is>
-          <t>Servicios: viáticos</t>
+          <t>Servicios: Viáticos</t>
         </is>
       </c>
       <c r="G16" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H16" s="16" t="inlineStr">
@@ -9111,12 +9111,12 @@
       </c>
       <c r="F17" s="18" t="inlineStr">
         <is>
-          <t>Servicios: viáticos</t>
+          <t>Servicios: Viáticos</t>
         </is>
       </c>
       <c r="G17" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H17" s="18" t="inlineStr">
@@ -9199,7 +9199,7 @@
       </c>
       <c r="G18" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H18" s="16" t="inlineStr">
@@ -9277,12 +9277,12 @@
       </c>
       <c r="F19" s="18" t="inlineStr">
         <is>
-          <t>Servicios: viáticos</t>
+          <t>Servicios: Viáticos</t>
         </is>
       </c>
       <c r="G19" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H19" s="18" t="inlineStr">
@@ -9365,7 +9365,7 @@
       </c>
       <c r="G20" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H20" s="16" t="inlineStr">
@@ -9452,7 +9452,7 @@
       </c>
       <c r="G21" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H21" s="18" t="inlineStr">
@@ -9539,7 +9539,7 @@
       </c>
       <c r="G22" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H22" s="16" t="inlineStr">
@@ -9626,7 +9626,7 @@
       </c>
       <c r="G23" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H23" s="18" t="inlineStr">
@@ -9708,12 +9708,12 @@
       </c>
       <c r="F24" s="16" t="inlineStr">
         <is>
-          <t>Servicios: viáticos</t>
+          <t>Servicios: Viáticos</t>
         </is>
       </c>
       <c r="G24" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H24" s="16" t="inlineStr">
@@ -9796,7 +9796,7 @@
       </c>
       <c r="G25" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H25" s="18" t="inlineStr">
@@ -9883,7 +9883,7 @@
       </c>
       <c r="G26" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H26" s="16" t="inlineStr">
@@ -9970,7 +9970,7 @@
       </c>
       <c r="G27" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H27" s="18" t="inlineStr">
@@ -10057,7 +10057,7 @@
       </c>
       <c r="G28" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H28" s="16" t="inlineStr">
@@ -10144,7 +10144,7 @@
       </c>
       <c r="G29" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H29" s="18" t="inlineStr">
@@ -10231,7 +10231,7 @@
       </c>
       <c r="G30" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H30" s="16" t="inlineStr">
@@ -10318,7 +10318,7 @@
       </c>
       <c r="G31" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H31" s="18" t="inlineStr">
@@ -10405,7 +10405,7 @@
       </c>
       <c r="G32" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H32" s="16" t="inlineStr">
@@ -10492,7 +10492,7 @@
       </c>
       <c r="G33" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H33" s="18" t="inlineStr">
@@ -10579,7 +10579,7 @@
       </c>
       <c r="G34" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H34" s="16" t="inlineStr">
@@ -10661,12 +10661,12 @@
       </c>
       <c r="F35" s="18" t="inlineStr">
         <is>
-          <t>Servicios: viáticos</t>
+          <t>Servicios: Viáticos</t>
         </is>
       </c>
       <c r="G35" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H35" s="18" t="inlineStr">
@@ -10749,7 +10749,7 @@
       </c>
       <c r="G36" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H36" s="16" t="inlineStr">
@@ -10836,7 +10836,7 @@
       </c>
       <c r="G37" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H37" s="18" t="inlineStr">
@@ -10923,7 +10923,7 @@
       </c>
       <c r="G38" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H38" s="16" t="inlineStr">
@@ -11010,7 +11010,7 @@
       </c>
       <c r="G39" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H39" s="18" t="inlineStr">
@@ -11088,12 +11088,12 @@
       </c>
       <c r="F40" s="16" t="inlineStr">
         <is>
-          <t>Servicios: viáticos</t>
+          <t>Servicios: Viáticos</t>
         </is>
       </c>
       <c r="G40" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H40" s="16" t="inlineStr">
@@ -11175,12 +11175,12 @@
       </c>
       <c r="F41" s="18" t="inlineStr">
         <is>
-          <t>Servicios: viáticos</t>
+          <t>Servicios: Viáticos</t>
         </is>
       </c>
       <c r="G41" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H41" s="18" t="inlineStr">
@@ -11267,7 +11267,7 @@
       </c>
       <c r="G42" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H42" s="16" t="inlineStr">
@@ -11349,12 +11349,12 @@
       </c>
       <c r="F43" s="18" t="inlineStr">
         <is>
-          <t>Servicios: viáticos</t>
+          <t>Servicios: Viáticos</t>
         </is>
       </c>
       <c r="G43" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H43" s="18" t="inlineStr">
@@ -11437,7 +11437,7 @@
       </c>
       <c r="G44" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H44" s="16" t="inlineStr">
@@ -11519,12 +11519,12 @@
       </c>
       <c r="F45" s="18" t="inlineStr">
         <is>
-          <t>Servicios: viáticos</t>
+          <t>Servicios: Viáticos</t>
         </is>
       </c>
       <c r="G45" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H45" s="18" t="inlineStr">
@@ -11607,7 +11607,7 @@
       </c>
       <c r="G46" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H46" s="16" t="inlineStr">
@@ -11689,12 +11689,12 @@
       </c>
       <c r="F47" s="18" t="inlineStr">
         <is>
-          <t>Servicios: viáticos</t>
+          <t>Servicios: Viáticos</t>
         </is>
       </c>
       <c r="G47" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H47" s="18" t="inlineStr">
@@ -11776,12 +11776,12 @@
       </c>
       <c r="F48" s="16" t="inlineStr">
         <is>
-          <t>Servicios: viáticos</t>
+          <t>Servicios: Viáticos</t>
         </is>
       </c>
       <c r="G48" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H48" s="16" t="inlineStr">
@@ -11868,7 +11868,7 @@
       </c>
       <c r="G49" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H49" s="18" t="inlineStr">
@@ -11951,7 +11951,7 @@
       </c>
       <c r="G50" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H50" s="16" t="inlineStr">
@@ -12038,7 +12038,7 @@
       </c>
       <c r="G51" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H51" s="18" t="inlineStr">
@@ -12121,7 +12121,7 @@
       </c>
       <c r="G52" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H52" s="16" t="inlineStr">
@@ -12208,7 +12208,7 @@
       </c>
       <c r="G53" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H53" s="18" t="inlineStr">
@@ -12295,7 +12295,7 @@
       </c>
       <c r="G54" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H54" s="16" t="inlineStr">
@@ -12382,7 +12382,7 @@
       </c>
       <c r="G55" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H55" s="18" t="inlineStr">
@@ -12469,7 +12469,7 @@
       </c>
       <c r="G56" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H56" s="16" t="inlineStr">
@@ -12556,7 +12556,7 @@
       </c>
       <c r="G57" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H57" s="18" t="inlineStr">
@@ -12643,7 +12643,7 @@
       </c>
       <c r="G58" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H58" s="16" t="inlineStr">
@@ -12730,7 +12730,7 @@
       </c>
       <c r="G59" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H59" s="18" t="inlineStr">
@@ -12817,7 +12817,7 @@
       </c>
       <c r="G60" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H60" s="16" t="inlineStr">
@@ -12904,7 +12904,7 @@
       </c>
       <c r="G61" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H61" s="18" t="inlineStr">
@@ -12991,7 +12991,7 @@
       </c>
       <c r="G62" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H62" s="16" t="inlineStr">
@@ -13078,7 +13078,7 @@
       </c>
       <c r="G63" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H63" s="18" t="inlineStr">
@@ -13165,7 +13165,7 @@
       </c>
       <c r="G64" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H64" s="16" t="inlineStr">
@@ -13252,7 +13252,7 @@
       </c>
       <c r="G65" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H65" s="18" t="inlineStr">
@@ -13339,7 +13339,7 @@
       </c>
       <c r="G66" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H66" s="16" t="inlineStr">
@@ -13426,7 +13426,7 @@
       </c>
       <c r="G67" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H67" s="18" t="inlineStr">
@@ -13513,7 +13513,7 @@
       </c>
       <c r="G68" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H68" s="16" t="inlineStr">
@@ -13600,7 +13600,7 @@
       </c>
       <c r="G69" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H69" s="18" t="inlineStr">
@@ -13687,7 +13687,7 @@
       </c>
       <c r="G70" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H70" s="16" t="inlineStr">
@@ -13774,7 +13774,7 @@
       </c>
       <c r="G71" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H71" s="18" t="inlineStr">
@@ -13861,7 +13861,7 @@
       </c>
       <c r="G72" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H72" s="16" t="inlineStr">
@@ -13948,7 +13948,7 @@
       </c>
       <c r="G73" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H73" s="18" t="inlineStr">
@@ -14035,7 +14035,7 @@
       </c>
       <c r="G74" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H74" s="16" t="inlineStr">
@@ -14122,7 +14122,7 @@
       </c>
       <c r="G75" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H75" s="18" t="inlineStr">
@@ -14209,7 +14209,7 @@
       </c>
       <c r="G76" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H76" s="16" t="inlineStr">
@@ -14296,7 +14296,7 @@
       </c>
       <c r="G77" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H77" s="18" t="inlineStr">
@@ -14383,7 +14383,7 @@
       </c>
       <c r="G78" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H78" s="16" t="inlineStr">
@@ -14470,7 +14470,7 @@
       </c>
       <c r="G79" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H79" s="18" t="inlineStr">
@@ -14557,7 +14557,7 @@
       </c>
       <c r="G80" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H80" s="16" t="inlineStr">
@@ -14644,7 +14644,7 @@
       </c>
       <c r="G81" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H81" s="18" t="inlineStr">
@@ -14731,7 +14731,7 @@
       </c>
       <c r="G82" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H82" s="16" t="inlineStr">
@@ -14818,7 +14818,7 @@
       </c>
       <c r="G83" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H83" s="18" t="inlineStr">
@@ -14905,7 +14905,7 @@
       </c>
       <c r="G84" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H84" s="16" t="inlineStr">
@@ -14992,7 +14992,7 @@
       </c>
       <c r="G85" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H85" s="18" t="inlineStr">
@@ -15079,7 +15079,7 @@
       </c>
       <c r="G86" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H86" s="16" t="inlineStr">
@@ -15166,7 +15166,7 @@
       </c>
       <c r="G87" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H87" s="18" t="inlineStr">
@@ -15253,7 +15253,7 @@
       </c>
       <c r="G88" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H88" s="16" t="inlineStr">
@@ -15335,12 +15335,12 @@
       </c>
       <c r="F89" s="18" t="inlineStr">
         <is>
-          <t>Servicios: viáticos</t>
+          <t>Servicios: Viáticos</t>
         </is>
       </c>
       <c r="G89" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H89" s="18" t="inlineStr">
@@ -15422,12 +15422,12 @@
       </c>
       <c r="F90" s="16" t="inlineStr">
         <is>
-          <t>Servicios: viáticos</t>
+          <t>Servicios: Viáticos</t>
         </is>
       </c>
       <c r="G90" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H90" s="16" t="inlineStr">
@@ -15514,7 +15514,7 @@
       </c>
       <c r="G91" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H91" s="18" t="inlineStr">
@@ -15592,12 +15592,12 @@
       </c>
       <c r="F92" s="16" t="inlineStr">
         <is>
-          <t>Servicios: viáticos</t>
+          <t>Servicios: Viáticos</t>
         </is>
       </c>
       <c r="G92" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H92" s="16" t="inlineStr">
@@ -15680,7 +15680,7 @@
       </c>
       <c r="G93" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H93" s="18" t="inlineStr">
@@ -15767,7 +15767,7 @@
       </c>
       <c r="G94" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H94" s="16" t="inlineStr">
@@ -15854,7 +15854,7 @@
       </c>
       <c r="G95" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H95" s="18" t="inlineStr">
@@ -15937,7 +15937,7 @@
       </c>
       <c r="G96" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H96" s="16" t="inlineStr">
@@ -16024,7 +16024,7 @@
       </c>
       <c r="G97" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H97" s="18" t="inlineStr">
@@ -16459,7 +16459,7 @@
       </c>
       <c r="G102" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H102" s="16" t="inlineStr">
@@ -16546,7 +16546,7 @@
       </c>
       <c r="G103" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H103" s="18" t="inlineStr">
@@ -16633,7 +16633,7 @@
       </c>
       <c r="G104" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H104" s="16" t="inlineStr">
@@ -16720,7 +16720,7 @@
       </c>
       <c r="G105" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H105" s="18" t="inlineStr">
@@ -16807,7 +16807,7 @@
       </c>
       <c r="G106" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H106" s="16" t="inlineStr">
@@ -16894,7 +16894,7 @@
       </c>
       <c r="G107" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H107" s="18" t="inlineStr">
@@ -16981,7 +16981,7 @@
       </c>
       <c r="G108" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H108" s="16" t="inlineStr">
@@ -17068,7 +17068,7 @@
       </c>
       <c r="G109" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H109" s="18" t="inlineStr">
@@ -17238,7 +17238,7 @@
       </c>
       <c r="G111" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H111" s="18" t="inlineStr">
@@ -17325,7 +17325,7 @@
       </c>
       <c r="G112" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H112" s="16" t="inlineStr">
@@ -17412,7 +17412,7 @@
       </c>
       <c r="G113" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H113" s="18" t="inlineStr">
@@ -17499,7 +17499,7 @@
       </c>
       <c r="G114" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H114" s="16" t="inlineStr">
@@ -17586,7 +17586,7 @@
       </c>
       <c r="G115" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H115" s="18" t="inlineStr">
@@ -17673,7 +17673,7 @@
       </c>
       <c r="G116" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H116" s="16" t="inlineStr">
@@ -17760,7 +17760,7 @@
       </c>
       <c r="G117" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H117" s="18" t="inlineStr">
@@ -17847,7 +17847,7 @@
       </c>
       <c r="G118" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H118" s="16" t="inlineStr">
@@ -17934,7 +17934,7 @@
       </c>
       <c r="G119" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H119" s="18" t="inlineStr">
@@ -18021,7 +18021,7 @@
       </c>
       <c r="G120" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H120" s="16" t="inlineStr">
@@ -18108,7 +18108,7 @@
       </c>
       <c r="G121" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H121" s="18" t="inlineStr">
@@ -18195,7 +18195,7 @@
       </c>
       <c r="G122" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H122" s="16" t="inlineStr">
@@ -18282,7 +18282,7 @@
       </c>
       <c r="G123" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H123" s="18" t="inlineStr">
@@ -18369,7 +18369,7 @@
       </c>
       <c r="G124" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H124" s="16" t="inlineStr">
@@ -18456,7 +18456,7 @@
       </c>
       <c r="G125" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H125" s="18" t="inlineStr">
@@ -18543,7 +18543,7 @@
       </c>
       <c r="G126" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H126" s="16" t="inlineStr">
@@ -18630,7 +18630,7 @@
       </c>
       <c r="G127" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H127" s="18" t="inlineStr">
@@ -18717,7 +18717,7 @@
       </c>
       <c r="G128" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H128" s="16" t="inlineStr">
@@ -18804,7 +18804,7 @@
       </c>
       <c r="G129" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H129" s="18" t="inlineStr">
@@ -18891,7 +18891,7 @@
       </c>
       <c r="G130" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H130" s="16" t="inlineStr">
@@ -18978,7 +18978,7 @@
       </c>
       <c r="G131" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H131" s="18" t="inlineStr">
@@ -19065,7 +19065,7 @@
       </c>
       <c r="G132" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H132" s="16" t="inlineStr">
@@ -19152,7 +19152,7 @@
       </c>
       <c r="G133" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H133" s="18" t="inlineStr">
@@ -19239,7 +19239,7 @@
       </c>
       <c r="G134" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H134" s="16" t="inlineStr">
@@ -19326,7 +19326,7 @@
       </c>
       <c r="G135" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H135" s="18" t="inlineStr">
@@ -19413,7 +19413,7 @@
       </c>
       <c r="G136" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H136" s="16" t="inlineStr">
@@ -19500,7 +19500,7 @@
       </c>
       <c r="G137" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H137" s="18" t="inlineStr">
@@ -19587,7 +19587,7 @@
       </c>
       <c r="G138" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H138" s="16" t="inlineStr">
@@ -19674,7 +19674,7 @@
       </c>
       <c r="G139" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H139" s="18" t="inlineStr">
@@ -19761,7 +19761,7 @@
       </c>
       <c r="G140" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H140" s="16" t="inlineStr">
@@ -19848,7 +19848,7 @@
       </c>
       <c r="G141" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H141" s="18" t="inlineStr">
@@ -19935,7 +19935,7 @@
       </c>
       <c r="G142" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H142" s="16" t="inlineStr">
@@ -20022,7 +20022,7 @@
       </c>
       <c r="G143" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H143" s="18" t="inlineStr">
@@ -20109,7 +20109,7 @@
       </c>
       <c r="G144" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H144" s="16" t="inlineStr">
@@ -20196,7 +20196,7 @@
       </c>
       <c r="G145" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H145" s="18" t="inlineStr">
@@ -20283,7 +20283,7 @@
       </c>
       <c r="G146" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H146" s="16" t="inlineStr">
@@ -20370,7 +20370,7 @@
       </c>
       <c r="G147" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H147" s="18" t="inlineStr">
@@ -20457,7 +20457,7 @@
       </c>
       <c r="G148" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H148" s="16" t="inlineStr">
@@ -20544,7 +20544,7 @@
       </c>
       <c r="G149" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H149" s="18" t="inlineStr">
@@ -20631,7 +20631,7 @@
       </c>
       <c r="G150" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H150" s="16" t="inlineStr">
@@ -20718,7 +20718,7 @@
       </c>
       <c r="G151" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H151" s="18" t="inlineStr">
@@ -20805,7 +20805,7 @@
       </c>
       <c r="G152" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H152" s="16" t="inlineStr">
@@ -20892,7 +20892,7 @@
       </c>
       <c r="G153" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H153" s="18" t="inlineStr">
@@ -20979,7 +20979,7 @@
       </c>
       <c r="G154" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H154" s="16" t="inlineStr">
@@ -21066,7 +21066,7 @@
       </c>
       <c r="G155" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H155" s="18" t="inlineStr">
@@ -21153,7 +21153,7 @@
       </c>
       <c r="G156" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H156" s="16" t="inlineStr">
@@ -21240,7 +21240,7 @@
       </c>
       <c r="G157" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H157" s="18" t="inlineStr">
@@ -21327,7 +21327,7 @@
       </c>
       <c r="G158" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H158" s="16" t="inlineStr">
@@ -21414,7 +21414,7 @@
       </c>
       <c r="G159" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H159" s="18" t="inlineStr">
@@ -21501,7 +21501,7 @@
       </c>
       <c r="G160" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H160" s="16" t="inlineStr">
@@ -21588,7 +21588,7 @@
       </c>
       <c r="G161" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H161" s="18" t="inlineStr">
@@ -21675,7 +21675,7 @@
       </c>
       <c r="G162" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H162" s="16" t="inlineStr">
@@ -21762,7 +21762,7 @@
       </c>
       <c r="G163" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H163" s="18" t="inlineStr">
@@ -21849,7 +21849,7 @@
       </c>
       <c r="G164" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H164" s="16" t="inlineStr">
@@ -21936,7 +21936,7 @@
       </c>
       <c r="G165" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H165" s="18" t="inlineStr">
@@ -22023,7 +22023,7 @@
       </c>
       <c r="G166" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H166" s="16" t="inlineStr">
@@ -22110,7 +22110,7 @@
       </c>
       <c r="G167" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H167" s="18" t="inlineStr">
@@ -22197,7 +22197,7 @@
       </c>
       <c r="G168" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H168" s="16" t="inlineStr">
@@ -22284,7 +22284,7 @@
       </c>
       <c r="G169" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H169" s="18" t="inlineStr">
@@ -22371,7 +22371,7 @@
       </c>
       <c r="G170" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H170" s="16" t="inlineStr">
@@ -22458,7 +22458,7 @@
       </c>
       <c r="G171" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H171" s="18" t="inlineStr">
@@ -22545,7 +22545,7 @@
       </c>
       <c r="G172" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H172" s="16" t="inlineStr">
@@ -22632,7 +22632,7 @@
       </c>
       <c r="G173" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H173" s="18" t="inlineStr">
@@ -22719,7 +22719,7 @@
       </c>
       <c r="G174" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H174" s="16" t="inlineStr">
@@ -22806,7 +22806,7 @@
       </c>
       <c r="G175" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H175" s="18" t="inlineStr">
@@ -22893,7 +22893,7 @@
       </c>
       <c r="G176" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H176" s="16" t="inlineStr">
@@ -22980,7 +22980,7 @@
       </c>
       <c r="G177" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H177" s="18" t="inlineStr">
@@ -23067,7 +23067,7 @@
       </c>
       <c r="G178" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H178" s="16" t="inlineStr">
@@ -23154,7 +23154,7 @@
       </c>
       <c r="G179" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H179" s="18" t="inlineStr">
@@ -23241,7 +23241,7 @@
       </c>
       <c r="G180" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H180" s="16" t="inlineStr">
@@ -23328,7 +23328,7 @@
       </c>
       <c r="G181" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H181" s="18" t="inlineStr">
@@ -23415,7 +23415,7 @@
       </c>
       <c r="G182" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H182" s="16" t="inlineStr">
@@ -23502,7 +23502,7 @@
       </c>
       <c r="G183" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H183" s="18" t="inlineStr">
@@ -23589,7 +23589,7 @@
       </c>
       <c r="G184" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H184" s="16" t="inlineStr">
@@ -23676,7 +23676,7 @@
       </c>
       <c r="G185" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H185" s="18" t="inlineStr">
@@ -23763,7 +23763,7 @@
       </c>
       <c r="G186" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H186" s="16" t="inlineStr">
@@ -23850,7 +23850,7 @@
       </c>
       <c r="G187" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H187" s="18" t="inlineStr">
@@ -23937,7 +23937,7 @@
       </c>
       <c r="G188" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H188" s="16" t="inlineStr">
@@ -24024,7 +24024,7 @@
       </c>
       <c r="G189" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H189" s="18" t="inlineStr">
@@ -24111,7 +24111,7 @@
       </c>
       <c r="G190" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H190" s="16" t="inlineStr">
@@ -24198,7 +24198,7 @@
       </c>
       <c r="G191" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H191" s="18" t="inlineStr">
@@ -24285,7 +24285,7 @@
       </c>
       <c r="G192" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H192" s="16" t="inlineStr">
@@ -24372,7 +24372,7 @@
       </c>
       <c r="G193" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H193" s="18" t="inlineStr">
@@ -24459,7 +24459,7 @@
       </c>
       <c r="G194" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H194" s="16" t="inlineStr">
@@ -24546,7 +24546,7 @@
       </c>
       <c r="G195" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H195" s="18" t="inlineStr">
@@ -24633,7 +24633,7 @@
       </c>
       <c r="G196" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H196" s="16" t="inlineStr">
@@ -24720,7 +24720,7 @@
       </c>
       <c r="G197" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H197" s="18" t="inlineStr">
@@ -24807,7 +24807,7 @@
       </c>
       <c r="G198" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H198" s="16" t="inlineStr">
@@ -24894,7 +24894,7 @@
       </c>
       <c r="G199" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H199" s="18" t="inlineStr">
@@ -24981,7 +24981,7 @@
       </c>
       <c r="G200" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H200" s="16" t="inlineStr">
@@ -25068,7 +25068,7 @@
       </c>
       <c r="G201" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H201" s="18" t="inlineStr">
@@ -25155,7 +25155,7 @@
       </c>
       <c r="G202" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H202" s="16" t="inlineStr">
@@ -25242,7 +25242,7 @@
       </c>
       <c r="G203" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H203" s="18" t="inlineStr">
@@ -25329,7 +25329,7 @@
       </c>
       <c r="G204" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H204" s="16" t="inlineStr">
@@ -25412,7 +25412,7 @@
       </c>
       <c r="G205" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H205" s="18" t="inlineStr">
@@ -25499,7 +25499,7 @@
       </c>
       <c r="G206" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H206" s="16" t="inlineStr">
@@ -25586,7 +25586,7 @@
       </c>
       <c r="G207" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H207" s="18" t="inlineStr">
@@ -25673,7 +25673,7 @@
       </c>
       <c r="G208" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H208" s="16" t="inlineStr">
@@ -25760,7 +25760,7 @@
       </c>
       <c r="G209" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H209" s="18" t="inlineStr">
@@ -25847,7 +25847,7 @@
       </c>
       <c r="G210" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H210" s="16" t="inlineStr">
@@ -25934,7 +25934,7 @@
       </c>
       <c r="G211" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H211" s="18" t="inlineStr">
@@ -26021,7 +26021,7 @@
       </c>
       <c r="G212" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H212" s="16" t="inlineStr">
@@ -26108,7 +26108,7 @@
       </c>
       <c r="G213" s="18" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H213" s="18" t="inlineStr">
@@ -26195,7 +26195,7 @@
       </c>
       <c r="G214" s="16" t="inlineStr">
         <is>
-          <t>(sin subgrupo)</t>
+          <t>(Sin Subgrupo)</t>
         </is>
       </c>
       <c r="H214" s="16" t="inlineStr">

</xml_diff>